<commit_message>
Peso por unidad: resueltas 43854 de 87836 filas (huevo, pan, galleta salada, cebolla roja, ajo) con fuentes citadas (USDA, UMPIH, normas de gradacion)
</commit_message>
<xml_diff>
--- a/data/raw/data_raw_unidades.xlsx
+++ b/data/raw/data_raw_unidades.xlsx
@@ -2723,7 +2723,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H197"/>
+  <dimension ref="A1:H200"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="14.90625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -9443,6 +9443,99 @@
       <c r="H197" t="inlineStr">
         <is>
           <t>Sin unidad de presentación: el hogar reportó directamente en la unidad base, resuelta fila a fila en 01_import.R sin pasar por esta tabla.</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="n">
+        <v>15</v>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>HUEVOS</t>
+        </is>
+      </c>
+      <c r="C198" t="n">
+        <v>1</v>
+      </c>
+      <c r="D198" t="inlineStr">
+        <is>
+          <t>Unidad</t>
+        </is>
+      </c>
+      <c r="E198" t="n">
+        <v>53</v>
+      </c>
+      <c r="F198" t="inlineStr">
+        <is>
+          <t>ALTA_CONFIANZA_fuente_externa</t>
+        </is>
+      </c>
+      <c r="G198" t="inlineStr">
+        <is>
+          <t>Huevo mediano con cascara, ~53g. Fuente: normas de gradacion Argentina (SENASA Decreto 4238/68) y Colombia, consistentes entre si. Peso por unidad (2026-09-08).</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="n">
+        <v>1</v>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>PANES</t>
+        </is>
+      </c>
+      <c r="C199" t="n">
+        <v>1</v>
+      </c>
+      <c r="D199" t="inlineStr">
+        <is>
+          <t>Unidad</t>
+        </is>
+      </c>
+      <c r="E199" t="n">
+        <v>50</v>
+      </c>
+      <c r="F199" t="inlineStr">
+        <is>
+          <t>ALTA_CONFIANZA_fuente_externa</t>
+        </is>
+      </c>
+      <c r="G199" t="inlineStr">
+        <is>
+          <t>Pan sobado/pan de agua, ~50g por unidad. Fuente: UMPIH (RD) y estudio ProCompetencia 2017 sobre mercado del pan RD. Peso por unidad (2026-09-08).</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="n">
+        <v>3</v>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>GALLETAS SALADAS</t>
+        </is>
+      </c>
+      <c r="C200" t="n">
+        <v>1</v>
+      </c>
+      <c r="D200" t="inlineStr">
+        <is>
+          <t>Unidad</t>
+        </is>
+      </c>
+      <c r="E200" t="n">
+        <v>3</v>
+      </c>
+      <c r="F200" t="inlineStr">
+        <is>
+          <t>ALTA_CONFIANZA_fuente_externa</t>
+        </is>
+      </c>
+      <c r="G200" t="inlineStr">
+        <is>
+          <t>Galleta salada tipo saltine, ~3g por unidad. Fuente: USDA FoodData Central (saltine crackers, 5 galletas=15-16g). Peso por unidad (2026-09-08).</t>
         </is>
       </c>
     </row>
@@ -9473,7 +9566,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2009"/>
+  <dimension ref="A1:H2015"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -68655,6 +68748,174 @@
         </is>
       </c>
     </row>
+    <row r="2010">
+      <c r="B2010" t="inlineStr">
+        <is>
+          <t>Cebolla roja</t>
+        </is>
+      </c>
+      <c r="C2010" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2010" t="inlineStr">
+        <is>
+          <t>Unidad</t>
+        </is>
+      </c>
+      <c r="E2010" t="n">
+        <v>148</v>
+      </c>
+      <c r="G2010" t="inlineStr">
+        <is>
+          <t>ALTA_CONFIANZA_fuente_externa</t>
+        </is>
+      </c>
+      <c r="H2010" t="inlineStr">
+        <is>
+          <t>Cebolla roja mediana entera, con cascara, ~148g. Fuente: USDA FoodData Central (1 medium onion=148g). Peso por unidad (2026-09-08).</t>
+        </is>
+      </c>
+    </row>
+    <row r="2011">
+      <c r="B2011" t="inlineStr">
+        <is>
+          <t>Ajo</t>
+        </is>
+      </c>
+      <c r="C2011" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2011" t="inlineStr">
+        <is>
+          <t>Unidad</t>
+        </is>
+      </c>
+      <c r="E2011" t="n">
+        <v>3</v>
+      </c>
+      <c r="G2011" t="inlineStr">
+        <is>
+          <t>ALTA_CONFIANZA_fuente_externa</t>
+        </is>
+      </c>
+      <c r="H2011" t="inlineStr">
+        <is>
+          <t>Se asume 1 unidad = 1 diente de ajo, ~3g. Fuente: USDA FoodData Central (Garlic raw, FDC ID 169230: 1 clove=3g). Peso por unidad (2026-09-08).</t>
+        </is>
+      </c>
+    </row>
+    <row r="2012">
+      <c r="B2012" t="inlineStr">
+        <is>
+          <t>Huevos criollos (gallina)</t>
+        </is>
+      </c>
+      <c r="C2012" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2012" t="inlineStr">
+        <is>
+          <t>Unidad</t>
+        </is>
+      </c>
+      <c r="E2012" t="n">
+        <v>53</v>
+      </c>
+      <c r="G2012" t="inlineStr">
+        <is>
+          <t>ALTA_CONFIANZA_fuente_externa</t>
+        </is>
+      </c>
+      <c r="H2012" t="inlineStr">
+        <is>
+          <t>Huevo mediano con cascara, ~53g. Fuente: normas de gradacion Argentina/Colombia. Peso por unidad (2026-09-08).</t>
+        </is>
+      </c>
+    </row>
+    <row r="2013">
+      <c r="B2013" t="inlineStr">
+        <is>
+          <t>Huevos de granja (gallina)</t>
+        </is>
+      </c>
+      <c r="C2013" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2013" t="inlineStr">
+        <is>
+          <t>Unidad</t>
+        </is>
+      </c>
+      <c r="E2013" t="n">
+        <v>53</v>
+      </c>
+      <c r="G2013" t="inlineStr">
+        <is>
+          <t>ALTA_CONFIANZA_fuente_externa</t>
+        </is>
+      </c>
+      <c r="H2013" t="inlineStr">
+        <is>
+          <t>Mismo criterio que 'Huevos criollos'. Peso por unidad (2026-09-08).</t>
+        </is>
+      </c>
+    </row>
+    <row r="2014">
+      <c r="B2014" t="inlineStr">
+        <is>
+          <t>Pan de agua</t>
+        </is>
+      </c>
+      <c r="C2014" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2014" t="inlineStr">
+        <is>
+          <t>Unidad</t>
+        </is>
+      </c>
+      <c r="E2014" t="n">
+        <v>50</v>
+      </c>
+      <c r="G2014" t="inlineStr">
+        <is>
+          <t>ALTA_CONFIANZA_fuente_externa</t>
+        </is>
+      </c>
+      <c r="H2014" t="inlineStr">
+        <is>
+          <t>Fuente: UMPIH y ProCompetencia 2017 (mercado del pan RD). Peso por unidad (2026-09-08).</t>
+        </is>
+      </c>
+    </row>
+    <row r="2015">
+      <c r="B2015" t="inlineStr">
+        <is>
+          <t>Pan sobado</t>
+        </is>
+      </c>
+      <c r="C2015" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2015" t="inlineStr">
+        <is>
+          <t>Unidad</t>
+        </is>
+      </c>
+      <c r="E2015" t="n">
+        <v>50</v>
+      </c>
+      <c r="G2015" t="inlineStr">
+        <is>
+          <t>ALTA_CONFIANZA_fuente_externa</t>
+        </is>
+      </c>
+      <c r="H2015" t="inlineStr">
+        <is>
+          <t>Mismo criterio que 'Pan de agua'. Peso por unidad (2026-09-08).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Peso por unidad: Aji cubanela 288g, dato de campo propio (5 unidades=1440g). 52416/87836 filas resueltas (60%)
</commit_message>
<xml_diff>
--- a/data/raw/data_raw_unidades.xlsx
+++ b/data/raw/data_raw_unidades.xlsx
@@ -9566,7 +9566,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2015"/>
+  <dimension ref="A1:H2016"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -68916,6 +68916,34 @@
         </is>
       </c>
     </row>
+    <row r="2016">
+      <c r="B2016" t="inlineStr">
+        <is>
+          <t>Ají grande (cubanela)</t>
+        </is>
+      </c>
+      <c r="C2016" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2016" t="inlineStr">
+        <is>
+          <t>Unidad</t>
+        </is>
+      </c>
+      <c r="E2016" t="n">
+        <v>288</v>
+      </c>
+      <c r="G2016" t="inlineStr">
+        <is>
+          <t>ALTA_CONFIANZA_campo_propio</t>
+        </is>
+      </c>
+      <c r="H2016" t="inlineStr">
+        <is>
+          <t>288g por unidad. Fuente: pesaje propio en mercado (La Sirena/Nacional), 5 ajies = 1440g en pesa digital, foto en media/fotos_investigacion_mercado/aji_cubanela02-03.jpg. Peso por unidad (2026-09-09).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Corregido bug de columnas (join error); peso por unidad 60%; documentada especificacion de Santiago sobre escenarios de fortificacion (audio 2026-09-09)
</commit_message>
<xml_diff>
--- a/data/raw/data_raw_unidades.xlsx
+++ b/data/raw/data_raw_unidades.xlsx
@@ -9447,93 +9447,84 @@
       </c>
     </row>
     <row r="198">
-      <c r="A198" t="n">
-        <v>15</v>
-      </c>
-      <c r="B198" t="inlineStr">
+      <c r="C198" t="inlineStr">
         <is>
           <t>HUEVOS</t>
         </is>
       </c>
-      <c r="C198" t="n">
-        <v>1</v>
-      </c>
-      <c r="D198" t="inlineStr">
+      <c r="D198" t="n">
+        <v>1</v>
+      </c>
+      <c r="E198" t="inlineStr">
         <is>
           <t>Unidad</t>
         </is>
       </c>
-      <c r="E198" t="n">
+      <c r="F198" t="n">
         <v>53</v>
       </c>
-      <c r="F198" t="inlineStr">
+      <c r="G198" t="inlineStr">
         <is>
           <t>ALTA_CONFIANZA_fuente_externa</t>
         </is>
       </c>
-      <c r="G198" t="inlineStr">
+      <c r="H198" t="inlineStr">
         <is>
           <t>Huevo mediano con cascara, ~53g. Fuente: normas de gradacion Argentina (SENASA Decreto 4238/68) y Colombia, consistentes entre si. Peso por unidad (2026-09-08).</t>
         </is>
       </c>
     </row>
     <row r="199">
-      <c r="A199" t="n">
-        <v>1</v>
-      </c>
-      <c r="B199" t="inlineStr">
+      <c r="C199" t="inlineStr">
         <is>
           <t>PANES</t>
         </is>
       </c>
-      <c r="C199" t="n">
-        <v>1</v>
-      </c>
-      <c r="D199" t="inlineStr">
+      <c r="D199" t="n">
+        <v>1</v>
+      </c>
+      <c r="E199" t="inlineStr">
         <is>
           <t>Unidad</t>
         </is>
       </c>
-      <c r="E199" t="n">
+      <c r="F199" t="n">
         <v>50</v>
       </c>
-      <c r="F199" t="inlineStr">
+      <c r="G199" t="inlineStr">
         <is>
           <t>ALTA_CONFIANZA_fuente_externa</t>
         </is>
       </c>
-      <c r="G199" t="inlineStr">
+      <c r="H199" t="inlineStr">
         <is>
           <t>Pan sobado/pan de agua, ~50g por unidad. Fuente: UMPIH (RD) y estudio ProCompetencia 2017 sobre mercado del pan RD. Peso por unidad (2026-09-08).</t>
         </is>
       </c>
     </row>
     <row r="200">
-      <c r="A200" t="n">
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>GALLETAS SALADAS</t>
+        </is>
+      </c>
+      <c r="D200" t="n">
+        <v>1</v>
+      </c>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>Unidad</t>
+        </is>
+      </c>
+      <c r="F200" t="n">
         <v>3</v>
       </c>
-      <c r="B200" t="inlineStr">
-        <is>
-          <t>GALLETAS SALADAS</t>
-        </is>
-      </c>
-      <c r="C200" t="n">
-        <v>1</v>
-      </c>
-      <c r="D200" t="inlineStr">
-        <is>
-          <t>Unidad</t>
-        </is>
-      </c>
-      <c r="E200" t="n">
-        <v>3</v>
-      </c>
-      <c r="F200" t="inlineStr">
+      <c r="G200" t="inlineStr">
         <is>
           <t>ALTA_CONFIANZA_fuente_externa</t>
         </is>
       </c>
-      <c r="G200" t="inlineStr">
+      <c r="H200" t="inlineStr">
         <is>
           <t>Galleta salada tipo saltine, ~3g por unidad. Fuente: USDA FoodData Central (saltine crackers, 5 galletas=15-16g). Peso por unidad (2026-09-08).</t>
         </is>

</xml_diff>

<commit_message>
Corregir 2 bugs activos de joins y añadir checks de integridad de claves
1. Fan-out Sec 3A (17,698 filas duplicadas): las filas de peso-por-unidad
   del 08/09-09 duplicaban la clave (descripcion, unidad 1) con filas
   previas de Pan sobado (45g) y Ají cubanela (90.7g); el left_join
   duplicaba cada registro de esos alimentos. FC viejos retirados, valor
   original conservado en nota (principio 6).
2. Filas inertes Sec 2: HUEVOS/PANES/GALLETAS SALADAS (peso-por-unidad)
   tenían 'variedad' vacío y nunca se aplicaban (2,732 filas de HUEVOS a
   0% resuelto). Variedad y frecuencia llenadas. Sec 2 sin FC: 8,655 -> 4,413.
3. 01_import.R: verificar_claves_join() detiene el pipeline ante claves
   duplicadas o filas con FC y clave vacía (6 tablas verificadas).

Descubrimientos y evidencia: INFORME_AUDITORIA_2026-09-10.md

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/data/raw/data_raw_unidades.xlsx
+++ b/data/raw/data_raw_unidades.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="diccionario_unidades" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="diccionario_conversion" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cuest. B Sec 2" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cuest. B Sec 3A" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="diccionario_unidades" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="diccionario_conversion" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Cuest. B Sec 2" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Cuest. B Sec 3A" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Cuest. B Sec 2'!$B$1:$H$197</definedName>
@@ -9447,6 +9447,12 @@
       </c>
     </row>
     <row r="198">
+      <c r="A198" t="n">
+        <v>2637</v>
+      </c>
+      <c r="B198" t="n">
+        <v>15</v>
+      </c>
       <c r="C198" t="inlineStr">
         <is>
           <t>HUEVOS</t>
@@ -9475,6 +9481,12 @@
       </c>
     </row>
     <row r="199">
+      <c r="A199" t="n">
+        <v>1090</v>
+      </c>
+      <c r="B199" t="n">
+        <v>1</v>
+      </c>
       <c r="C199" t="inlineStr">
         <is>
           <t>PANES</t>
@@ -9503,6 +9515,12 @@
       </c>
     </row>
     <row r="200">
+      <c r="A200" t="n">
+        <v>515</v>
+      </c>
+      <c r="B200" t="n">
+        <v>3</v>
+      </c>
       <c r="C200" t="inlineStr">
         <is>
           <t>GALLETAS SALADAS</t>
@@ -30097,20 +30115,17 @@
           <t>Unidad</t>
         </is>
       </c>
-      <c r="E706" t="n">
-        <v>45</v>
-      </c>
       <c r="F706" t="n">
         <v>9</v>
       </c>
       <c r="G706" t="inlineStr">
         <is>
-          <t>ALTA_CONFIANZA</t>
+          <t>RETIRADO_duplicado_clave_2026-09-10</t>
         </is>
       </c>
       <c r="H706" t="inlineStr">
         <is>
-          <t>FC = mediana de contenido_empaque_presentacion (N=5 hogares, crudo Sec3A).</t>
+          <t>FC = mediana de contenido_empaque_presentacion (N=5 hogares, crudo Sec3A). | FC retirado 2026-09-10 (auditoría externa): esta fila duplicaba la clave (descripcion + unidad 1) con la fila de peso-por-unidad añadida 2026-09-08 (50g, UMPIH/ProCompetencia), lo que duplicaba silenciosamente cada registro de 'Pan sobado por unidad' en el left_join de 01_import.R (9,131 filas duplicadas). Valor original conservado: FC=45 (mediana crudo, N=9). El FC vigente es 50g.</t>
         </is>
       </c>
     </row>
@@ -36251,20 +36266,17 @@
           <t>Unidad</t>
         </is>
       </c>
-      <c r="E910" t="n">
-        <v>90.7</v>
-      </c>
       <c r="F910" t="n">
         <v>5</v>
       </c>
       <c r="G910" t="inlineStr">
         <is>
-          <t>ALTA_CONFIANZA</t>
+          <t>RETIRADO_duplicado_clave_2026-09-10</t>
         </is>
       </c>
       <c r="H910" t="inlineStr">
         <is>
-          <t>FC = mediana de contenido_empaque_presentacion (N=4 hogares, crudo Sec3A).</t>
+          <t>FC = mediana de contenido_empaque_presentacion (N=4 hogares, crudo Sec3A). | FC retirado 2026-09-10 (auditoría externa): esta fila duplicaba la clave (descripcion + unidad 1) con la fila de peso-por-unidad añadida 2026-09-09 (288g, pesaje de campo propio, 5 unidades=1440g), lo que duplicaba silenciosamente cada registro de 'Ají cubanela por unidad' en el left_join de 01_import.R (8,567 filas duplicadas). Valor original conservado: FC=90.7 (mediana crudo, N=5). El FC vigente es 288g.</t>
         </is>
       </c>
     </row>

</xml_diff>